<commit_message>
FIX: headcounts and revenue in excel
</commit_message>
<xml_diff>
--- a/exports/companies.xlsx
+++ b/exports/companies.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="3" documentId="8_{10CD4188-C72D-CC49-9926-94CAECCCC7F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{745ED1E0-BC16-1D40-9B33-A7C457CB1388}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="33600" windowHeight="21000" xr2:uid="{868B1461-C732-A44F-8CF7-BFE9C77D16CD}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="20500" xr2:uid="{868B1461-C732-A44F-8CF7-BFE9C77D16CD}"/>
   </bookViews>
   <sheets>
     <sheet name="companies" sheetId="1" r:id="rId1"/>
@@ -1782,6 +1782,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -2102,9 +2106,11 @@
   <dimension ref="A1:R37"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="7" max="7" width="23.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="23.6640625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="49" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.1640625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="28" customWidth="1"/>
+    <col min="15" max="16" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.2">
@@ -2704,7 +2710,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="1:18" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:18" ht="340" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>136</v>
       </c>
@@ -2854,7 +2860,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="16" spans="1:18" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:18" ht="340" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>166</v>
       </c>
@@ -2904,7 +2910,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:16" ht="356" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>177</v>
       </c>
@@ -2954,7 +2960,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:16" ht="340" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>188</v>
       </c>
@@ -3004,7 +3010,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:16" ht="102" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>198</v>
       </c>
@@ -3051,7 +3057,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:16" ht="340" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>207</v>
       </c>
@@ -3098,7 +3104,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:16" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:16" ht="340" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>217</v>
       </c>
@@ -3145,7 +3151,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:16" ht="340" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>226</v>
       </c>
@@ -3195,7 +3201,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:16" ht="340" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>236</v>
       </c>
@@ -3245,7 +3251,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:16" ht="340" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>247</v>
       </c>
@@ -3295,7 +3301,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:16" ht="323" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>257</v>
       </c>
@@ -3345,7 +3351,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:16" ht="372" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>267</v>
       </c>
@@ -3395,7 +3401,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:16" ht="323" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>278</v>
       </c>
@@ -3445,7 +3451,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:16" ht="306" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>288</v>
       </c>
@@ -3495,7 +3501,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:16" ht="340" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>298</v>
       </c>
@@ -3545,7 +3551,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:16" ht="372" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>308</v>
       </c>
@@ -3592,7 +3598,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="31" spans="1:16" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:16" ht="404" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>318</v>
       </c>
@@ -3642,7 +3648,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="1:16" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:16" ht="306" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>328</v>
       </c>
@@ -3689,7 +3695,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:16" ht="340" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>337</v>
       </c>
@@ -3739,7 +3745,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:16" ht="356" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>348</v>
       </c>
@@ -3789,7 +3795,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:16" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>358</v>
       </c>
@@ -3839,7 +3845,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:16" ht="306" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>370</v>
       </c>
@@ -3889,7 +3895,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:16" ht="323" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>380</v>
       </c>

</xml_diff>